<commit_message>
current changes excluding 70-export
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ChaitanyaRavindra\Documents\UiPath\ConocoPhillips-Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A488A9B2-4542-4D63-B100-D8011444304D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781C77F1-16EB-4ADC-8A9E-F1B0299AD955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="247">
   <si>
     <t>Name</t>
   </si>
@@ -449,15 +449,9 @@
     <t>List of fields which will be checked versus a specific confidence threshold. All new entries must have the "-Confidence" suffix</t>
   </si>
   <si>
-    <t>OtherConfidenceFields</t>
-  </si>
-  <si>
     <t>List of fields which will be checked versus a single confidence #:  Other-Confidence</t>
   </si>
   <si>
-    <t>other-Confidence</t>
-  </si>
-  <si>
     <t>AlwaysValidateClassification</t>
   </si>
   <si>
@@ -728,64 +722,61 @@
     <t>SettlementStatements</t>
   </si>
   <si>
+    <t>LogMessage_SettlementPostProcessing</t>
+  </si>
+  <si>
+    <t>Starting Settlement Post Processing</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_DateFailure</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_MandatoryFieldsFailure</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_LineAmountFailureMath</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_LineAmountFailureEmpty</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_AlreadySetFalse</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_SubtotalFailure</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_TotalFailure</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_SubtotalPass</t>
+  </si>
+  <si>
+    <t>LogMessage_SettlementPostProcessing_ConfidenceFieldsFailure</t>
+  </si>
+  <si>
+    <t>Meter Number,Meter Name,Production Date,Pressure Base,MCF,MMBTU</t>
+  </si>
+  <si>
+    <t>Meter Number-Confidence</t>
+  </si>
+  <si>
+    <t>Meter Name-Confidence</t>
+  </si>
+  <si>
+    <t>Production Date-Confidence</t>
+  </si>
+  <si>
+    <t>Pressure Base-Confidence</t>
+  </si>
+  <si>
+    <t>MCF-Confidence</t>
+  </si>
+  <si>
+    <t>MMBTU-Confidence</t>
+  </si>
+  <si>
     <t>True</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing</t>
-  </si>
-  <si>
-    <t>Starting Settlement Post Processing</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_DateFailure</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_MandatoryFieldsFailure</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_LineAmountFailureMath</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_LineAmountFailureEmpty</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_AlreadySetFalse</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_SubtotalFailure</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_TotalFailure</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_SubtotalPass</t>
-  </si>
-  <si>
-    <t>LogMessage_SettlementPostProcessing_ConfidenceFieldsFailure</t>
-  </si>
-  <si>
-    <t>Meter Number,Meter Name,Production Date,Pressure Base,MCF,MMBTU</t>
-  </si>
-  <si>
-    <t>BTU,Basis,Allocation Decimal,Gas Lift MCF,Gas Lift MMBTU1,Diverted Gas MCF,Diverted Gas MMBTU</t>
-  </si>
-  <si>
-    <t>Meter Number-Confidence</t>
-  </si>
-  <si>
-    <t>Meter Name-Confidence</t>
-  </si>
-  <si>
-    <t>Production Date-Confidence</t>
-  </si>
-  <si>
-    <t>Pressure Base-Confidence</t>
-  </si>
-  <si>
-    <t>MCF-Confidence</t>
-  </si>
-  <si>
-    <t>MMBTU-Confidence</t>
   </si>
 </sst>
 </file>
@@ -857,7 +848,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -868,7 +859,6 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1263,7 +1253,7 @@
         <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1358,58 +1348,58 @@
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B14" t="s">
+        <v>200</v>
+      </c>
+      <c r="C14" t="s">
         <v>202</v>
-      </c>
-      <c r="C14" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>155</v>
-      </c>
       <c r="C18" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1419,13 +1409,13 @@
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B21">
         <v>0.5</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1433,13 +1423,13 @@
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1447,13 +1437,13 @@
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>219</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>223</v>
-      </c>
       <c r="C25" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1464,10 +1454,10 @@
         <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C27" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1475,10 +1465,10 @@
         <v>36</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C28" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1486,10 +1476,10 @@
         <v>37</v>
       </c>
       <c r="B29" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C29" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1497,10 +1487,10 @@
         <v>113</v>
       </c>
       <c r="B30" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C30" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1508,10 +1498,10 @@
         <v>77</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C31" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1519,10 +1509,10 @@
         <v>78</v>
       </c>
       <c r="B32" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C32" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2597,13 +2587,13 @@
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B7">
         <v>99999</v>
       </c>
       <c r="C7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2630,7 +2620,7 @@
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -2702,7 +2692,7 @@
         <v>75</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2718,7 +2708,7 @@
         <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2726,7 +2716,7 @@
         <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2742,7 +2732,7 @@
         <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2782,7 +2772,7 @@
         <v>76</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2798,7 +2788,7 @@
         <v>58</v>
       </c>
       <c r="B32" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2814,7 +2804,7 @@
         <v>59</v>
       </c>
       <c r="B34" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2827,18 +2817,18 @@
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B37" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2859,18 +2849,18 @@
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2926,18 +2916,18 @@
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B51" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B52" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2966,10 +2956,10 @@
     </row>
     <row r="56" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B56" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2986,7 +2976,7 @@
         <v>100</v>
       </c>
       <c r="B59" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2995,7 +2985,7 @@
         <v>54</v>
       </c>
       <c r="B61" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3020,7 +3010,7 @@
         <v>31</v>
       </c>
       <c r="B65" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4043,10 +4033,10 @@
         <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
@@ -5090,7 +5080,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0B409EA-78AE-4EDC-AD3C-5E59FD94E42A}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="57.5703125" bestFit="1" customWidth="1"/>
@@ -5111,15 +5101,15 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B3" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B4" t="s">
         <v>122</v>
@@ -5127,7 +5117,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B5" t="s">
         <v>123</v>
@@ -5135,7 +5125,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B6" t="s">
         <v>124</v>
@@ -5143,7 +5133,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B7" t="s">
         <v>125</v>
@@ -5151,7 +5141,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B8" t="s">
         <v>126</v>
@@ -5159,7 +5149,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="B9" t="s">
         <v>127</v>
@@ -5167,7 +5157,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B10" t="s">
         <v>128</v>
@@ -5175,7 +5165,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B11" t="s">
         <v>129</v>
@@ -5183,7 +5173,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B13" t="s">
         <v>130</v>
@@ -5197,7 +5187,7 @@
         <v>132</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C16" t="s">
         <v>133</v>
@@ -5211,77 +5201,61 @@
         <v>135</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C18" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>137</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="C19" t="s">
-        <v>138</v>
-      </c>
+      <c r="B19" s="2"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="B21" s="6">
+        <v>240</v>
+      </c>
+      <c r="B21">
         <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="B22" s="6">
+        <v>241</v>
+      </c>
+      <c r="B22">
         <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="B23" s="6">
+        <v>242</v>
+      </c>
+      <c r="B23">
         <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B24" s="6">
+        <v>243</v>
+      </c>
+      <c r="B24">
         <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>248</v>
-      </c>
-      <c r="B25" s="6">
+        <v>244</v>
+      </c>
+      <c r="B25">
         <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>249</v>
-      </c>
-      <c r="B26" s="6">
+        <v>245</v>
+      </c>
+      <c r="B26">
         <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>139</v>
-      </c>
-      <c r="B27" s="6">
-        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -5313,15 +5287,15 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B4" t="s">
         <v>122</v>
@@ -5329,7 +5303,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B5" t="s">
         <v>123</v>
@@ -5337,7 +5311,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B6" t="s">
         <v>126</v>
@@ -5345,7 +5319,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B7" t="s">
         <v>128</v>
@@ -5353,15 +5327,15 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B10" t="s">
         <v>130</v>
@@ -5369,10 +5343,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C12" t="s">
         <v>131</v>
@@ -5380,10 +5354,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B13" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C13" t="s">
         <v>133</v>
@@ -5391,10 +5365,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B14" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C14" t="s">
         <v>134</v>
@@ -5402,10 +5376,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B15" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C15" t="s">
         <v>136</v>
@@ -5413,18 +5387,18 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B16" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B18">
         <v>50</v>
@@ -5432,7 +5406,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B19">
         <v>85</v>
@@ -5440,7 +5414,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B20">
         <v>50</v>
@@ -5526,44 +5500,44 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B6" t="b">
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C7" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
everything other than export
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ChaitanyaRavindra\Documents\UiPath\ConocoPhillips-Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781C77F1-16EB-4ADC-8A9E-F1B0299AD955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2968AC49-8B5F-46C0-9751-5DD61E375299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="246">
   <si>
     <t>Name</t>
   </si>
@@ -774,9 +774,6 @@
   </si>
   <si>
     <t>MMBTU-Confidence</t>
-  </si>
-  <si>
-    <t>True</t>
   </si>
 </sst>
 </file>
@@ -1363,7 +1360,7 @@
         <v>138</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>246</v>
+        <v>153</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>154</v>
@@ -1412,7 +1409,7 @@
         <v>168</v>
       </c>
       <c r="B21">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>169</v>

</xml_diff>

<commit_message>
without recent mock changes
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ChaitanyaRavindra\Documents\UiPath\ConocoPhillips-Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92676D51-013F-47DF-B79A-22E5DED73F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C54F0A88-1576-4FBB-A88F-BB9739864155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="268">
   <si>
     <t>Name</t>
   </si>
@@ -251,9 +251,6 @@
     <t>Presenting Validation Station for:</t>
   </si>
   <si>
-    <t>Data\Exports\</t>
-  </si>
-  <si>
     <t>Data\ReceiptsTraining\</t>
   </si>
   <si>
@@ -746,24 +743,12 @@
     <t>MMBTU-Confidence</t>
   </si>
   <si>
-    <t>Initsheet</t>
-  </si>
-  <si>
-    <t>01 Hiland-Hiland-Bakken</t>
-  </si>
-  <si>
-    <t>Data\Exports\Output.xlsx</t>
-  </si>
-  <si>
     <t>OutputFile</t>
   </si>
   <si>
     <t>ReportPath</t>
   </si>
   <si>
-    <t>Data\Exports\Report.xlsx</t>
-  </si>
-  <si>
     <t>ReportSheet</t>
   </si>
   <si>
@@ -792,9 +777,6 @@
   </si>
   <si>
     <t>ConocoPhillips Process End</t>
-  </si>
-  <si>
-    <t>Hello,&lt;br&gt;&lt;br&gt;The &lt;b&gt;Conocophillips&lt;/b&gt; process has started.&lt;br&gt;&lt;ul&gt;&lt;li&gt;&lt;b&gt;Start Time:&lt;/b&gt; {StartTime}&lt;/li&gt;&lt;li&gt;&lt;b&gt;Machine:&lt;/b&gt; {MachineName}&lt;/li&gt;&lt;li&gt;&lt;b&gt;Source Queue:&lt;/b&gt; {QueueName}&lt;/li&gt;&lt;/ul&gt;&lt;br&gt;Regards,&lt;br&gt;Accelirate</t>
   </si>
   <si>
     <t>OrchestratorQueueName</t>
@@ -836,6 +818,30 @@
     <t>Hello,
 Conocophillips process has ended at {EndTime}.
 Regards</t>
+  </si>
+  <si>
+    <t>True</t>
+  </si>
+  <si>
+    <t>C:\Users\ChaitanyaRavindra\Documents\UiPath\ConocoPhillips-Performer\Data\Exports\Output.xlsx</t>
+  </si>
+  <si>
+    <t>C:\Users\ChaitanyaRavindra\Documents\UiPath\ConocoPhillips-Performer\Data\Exports\Report.xlsx</t>
+  </si>
+  <si>
+    <t>C:\Users\ChaitanyaRavindra\Documents\UiPath\ConocoPhillips-Performer\Data\Exports\</t>
+  </si>
+  <si>
+    <t>MaxRetry</t>
+  </si>
+  <si>
+    <t>ProcessName</t>
+  </si>
+  <si>
+    <t>EXCEL</t>
+  </si>
+  <si>
+    <t>Hello,&lt;br&gt;&lt;br&gt;The &lt;b&gt;Conocophillips&lt;/b&gt; process has started.&lt;br&gt;&lt;ul&gt;&lt;li&gt;&lt;b&gt;Start Time:&lt;/b&gt; {StartTime}&lt;/li&gt;&lt;li&gt;&lt;b&gt;Source Queue:&lt;/b&gt; {QueueName}&lt;/li&gt;&lt;/ul&gt;&lt;br&gt;Regards,&lt;br&gt;Accelirate</t>
   </si>
 </sst>
 </file>
@@ -1240,7 +1246,7 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.85546875" customWidth="1"/>
-    <col min="2" max="2" width="70.140625" customWidth="1"/>
+    <col min="2" max="2" width="88.85546875" customWidth="1"/>
     <col min="3" max="3" width="131.7109375" customWidth="1"/>
     <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
@@ -1281,10 +1287,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1313,13 +1319,13 @@
     </row>
     <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1327,7 +1333,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>263</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -1338,7 +1344,7 @@
         <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
         <v>64</v>
@@ -1349,7 +1355,7 @@
         <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C6" t="s">
         <v>65</v>
@@ -1387,7 +1393,7 @@
         <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1395,77 +1401,77 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
         <v>86</v>
-      </c>
-      <c r="C13" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>200</v>
+      </c>
+      <c r="B14" t="s">
+        <v>199</v>
+      </c>
+      <c r="C14" t="s">
         <v>201</v>
-      </c>
-      <c r="B14" t="s">
-        <v>200</v>
-      </c>
-      <c r="C14" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>153</v>
+        <v>260</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>153</v>
+        <v>260</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1475,13 +1481,13 @@
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>167</v>
+      </c>
+      <c r="B21">
+        <v>0.7</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="B21">
-        <v>0.6</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1489,13 +1495,13 @@
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>195</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C23" t="s">
         <v>196</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="C23" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1503,13 +1509,13 @@
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>218</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C25" t="s">
         <v>219</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="C25" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1520,10 +1526,10 @@
         <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C27" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1531,10 +1537,10 @@
         <v>36</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C28" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1542,120 +1548,120 @@
         <v>37</v>
       </c>
       <c r="B29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C30" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B32" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C32" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>236</v>
-      </c>
-      <c r="B34" t="s">
-        <v>237</v>
-      </c>
-    </row>
+        <v>166</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B35" t="s">
-        <v>238</v>
+        <v>261</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B36" t="s">
-        <v>241</v>
+        <v>262</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="B37" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B39" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B40" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="B43" s="6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B45" t="s">
+        <v>266</v>
+      </c>
+    </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="47" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="48" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2678,62 +2684,62 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6">
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B7">
         <v>99999</v>
       </c>
       <c r="C7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B8">
         <v>30</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2741,24 +2747,31 @@
         <v>48</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B11">
+        <v>5</v>
+      </c>
+    </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
@@ -2802,10 +2815,10 @@
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2818,10 +2831,10 @@
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2837,7 +2850,7 @@
         <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2845,7 +2858,7 @@
         <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2861,7 +2874,7 @@
         <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2874,10 +2887,10 @@
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" t="s">
         <v>90</v>
-      </c>
-      <c r="B27" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2898,10 +2911,10 @@
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2917,7 +2930,7 @@
         <v>58</v>
       </c>
       <c r="B32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2933,7 +2946,7 @@
         <v>59</v>
       </c>
       <c r="B34" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2946,18 +2959,18 @@
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>208</v>
+      </c>
+      <c r="B36" t="s">
         <v>209</v>
-      </c>
-      <c r="B36" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>210</v>
+      </c>
+      <c r="B37" t="s">
         <v>211</v>
-      </c>
-      <c r="B37" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2978,134 +2991,134 @@
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="43" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B43" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>117</v>
+      </c>
+      <c r="B44" t="s">
         <v>118</v>
-      </c>
-      <c r="B44" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>92</v>
+      </c>
+      <c r="B46" t="s">
         <v>93</v>
-      </c>
-      <c r="B46" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>110</v>
+      </c>
+      <c r="B50" t="s">
         <v>111</v>
-      </c>
-      <c r="B50" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>191</v>
+      </c>
+      <c r="B51" t="s">
         <v>192</v>
-      </c>
-      <c r="B51" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>193</v>
+      </c>
+      <c r="B52" t="s">
         <v>194</v>
-      </c>
-      <c r="B52" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>100</v>
+      </c>
+      <c r="B53" t="s">
         <v>101</v>
-      </c>
-      <c r="B53" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>104</v>
+      </c>
+      <c r="B54" t="s">
         <v>105</v>
-      </c>
-      <c r="B54" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>197</v>
+      </c>
+      <c r="B56" t="s">
         <v>198</v>
-      </c>
-      <c r="B56" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>97</v>
+      </c>
+      <c r="B58" t="s">
         <v>98</v>
-      </c>
-      <c r="B58" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B59" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3114,7 +3127,7 @@
         <v>54</v>
       </c>
       <c r="B61" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3139,7 +3152,7 @@
         <v>31</v>
       </c>
       <c r="B65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4162,10 +4175,10 @@
         <v>40</v>
       </c>
       <c r="B2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C2" t="s">
         <v>223</v>
-      </c>
-      <c r="C2" t="s">
-        <v>224</v>
       </c>
       <c r="D2" t="s">
         <v>38</v>
@@ -5230,82 +5243,82 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="B7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="B9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="B11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -5313,13 +5326,13 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>131</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C16" t="s">
         <v>132</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="C16" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -5327,13 +5340,13 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C18" t="s">
         <v>135</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="C18" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -5341,7 +5354,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B21">
         <v>80</v>
@@ -5349,7 +5362,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B22">
         <v>80</v>
@@ -5357,7 +5370,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B23">
         <v>80</v>
@@ -5365,7 +5378,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B24">
         <v>80</v>
@@ -5373,7 +5386,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B25">
         <v>80</v>
@@ -5381,7 +5394,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B26">
         <v>80</v>
@@ -5416,118 +5429,118 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" t="s">
         <v>170</v>
-      </c>
-      <c r="B3" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8" t="s">
         <v>176</v>
-      </c>
-      <c r="B8" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B12" t="s">
         <v>179</v>
       </c>
-      <c r="B12" t="s">
-        <v>180</v>
-      </c>
       <c r="C12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" t="s">
         <v>181</v>
       </c>
-      <c r="B13" t="s">
-        <v>182</v>
-      </c>
       <c r="C13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B14" t="s">
         <v>183</v>
       </c>
-      <c r="B14" t="s">
-        <v>184</v>
-      </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" t="s">
         <v>185</v>
       </c>
-      <c r="B15" t="s">
-        <v>186</v>
-      </c>
       <c r="C15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>186</v>
+      </c>
+      <c r="B16" t="s">
         <v>187</v>
       </c>
-      <c r="B16" t="s">
-        <v>188</v>
-      </c>
       <c r="C16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B18">
         <v>50</v>
@@ -5535,7 +5548,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B19">
         <v>85</v>
@@ -5543,7 +5556,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B20">
         <v>50</v>
@@ -5629,44 +5642,44 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C3" t="s">
         <v>203</v>
-      </c>
-      <c r="B3" t="s">
-        <v>216</v>
-      </c>
-      <c r="C3" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B6" t="b">
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>216</v>
+      </c>
+      <c r="C7" t="s">
         <v>217</v>
-      </c>
-      <c r="C7" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>